<commit_message>
test(contratos): regenerar las cohortes HTTP del review de catalogos
</commit_message>
<xml_diff>
--- a/src/test/fixtures/catalogs-http/imports/en/export.xlsx
+++ b/src/test/fixtures/catalogs-http/imports/en/export.xlsx
@@ -40,6 +40,9 @@
   </x:si>
   <x:si>
     <x:t>Uno cambiado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>One</x:t>
   </x:si>
   <x:si>
     <x:t>Yes</x:t>
@@ -477,61 +480,64 @@
       <x:c r="B2" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
       <x:c r="A3" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
       <x:c r="A4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
         <x:v>13</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
       <x:c r="A5" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:6">
       <x:c r="A6" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(fixtures): ejemplos HTTP de la exportación conjunta del cierre de Catálogos E2
Corrida 20261025-233355-14e4887e74f04628a4ea0748e3e0c988: dotnet test completo con
Docker en verde y 23 cohortes copiadas por el exportador, sin editar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/test/fixtures/catalogs-http/imports/en/export.xlsx
+++ b/src/test/fixtures/catalogs-http/imports/en/export.xlsx
@@ -24,13 +24,13 @@
     <x:t>Text</x:t>
   </x:si>
   <x:si>
-    <x:t>English text</x:t>
+    <x:t>Spanish text</x:t>
   </x:si>
   <x:si>
     <x:t>Detail</x:t>
   </x:si>
   <x:si>
-    <x:t>English detail</x:t>
+    <x:t>Spanish detail</x:t>
   </x:si>
   <x:si>
     <x:t>Active</x:t>
@@ -42,7 +42,7 @@
     <x:t>Uno cambiado</x:t>
   </x:si>
   <x:si>
-    <x:t>One</x:t>
+    <x:t>Uno</x:t>
   </x:si>
   <x:si>
     <x:t>Yes</x:t>
@@ -51,31 +51,31 @@
     <x:t>B</x:t>
   </x:si>
   <x:si>
+    <x:t>Two</x:t>
+  </x:si>
+  <x:si>
     <x:t>Dos</x:t>
   </x:si>
   <x:si>
-    <x:t>Two</x:t>
-  </x:si>
-  <x:si>
     <x:t>No</x:t>
   </x:si>
   <x:si>
     <x:t>C</x:t>
   </x:si>
   <x:si>
+    <x:t>Three</x:t>
+  </x:si>
+  <x:si>
     <x:t>Tres</x:t>
   </x:si>
   <x:si>
-    <x:t>Three</x:t>
-  </x:si>
-  <x:si>
     <x:t>D</x:t>
   </x:si>
   <x:si>
+    <x:t>Inactive</x:t>
+  </x:si>
+  <x:si>
     <x:t>Inactiva</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Inactive</x:t>
   </x:si>
   <x:si>
     <x:t>NEW</x:t>

</xml_diff>